<commit_message>
Configuración inicial del entorno frontend
- Configuración inicial del proyecto web con Angular.
- Configuración inicial del proyecto móvil con Ionic y Angular.
- Integración de Capacitor y plataforma Android.
- Configuración del lector QR.
- Ajuste de minSdkVersion a 26.
- Incorporación de README con versiones e instrucciones de configuración.
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Gantt CAPSTONE - SISTEMA DE GESTION PARA TRANSPORTE DE PASAJEROS.xlsx
+++ b/FASE 1/Evidencias Grupales/Gantt CAPSTONE - SISTEMA DE GESTION PARA TRANSPORTE DE PASAJEROS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\capstone-2026\FASE 1\Evidencias Grupales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D359EA11-FBC8-4DB0-9717-541D973AE0CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F2D6D62-C6AA-42AB-98FC-90DDF8999846}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gestión Proyecto Carta Gantt" sheetId="3" r:id="rId1"/>
@@ -1456,90 +1456,6 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="13" fillId="9" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1595,6 +1511,90 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1897,93 +1897,93 @@
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
-      <c r="I7" s="72"/>
-      <c r="J7" s="73"/>
-      <c r="K7" s="73"/>
-      <c r="L7" s="73"/>
-      <c r="M7" s="73"/>
-      <c r="N7" s="73"/>
-      <c r="O7" s="73"/>
-      <c r="P7" s="73"/>
-      <c r="Q7" s="73"/>
-      <c r="R7" s="73"/>
-      <c r="S7" s="73"/>
-      <c r="T7" s="73"/>
-      <c r="U7" s="73"/>
-      <c r="V7" s="73"/>
-      <c r="W7" s="73"/>
-      <c r="X7" s="73"/>
-      <c r="Y7" s="73"/>
-      <c r="Z7" s="73"/>
-      <c r="AA7" s="73"/>
-      <c r="AB7" s="74"/>
-      <c r="AC7" s="75"/>
-      <c r="AD7" s="76"/>
-      <c r="AE7" s="76"/>
-      <c r="AF7" s="76"/>
-      <c r="AG7" s="76"/>
-      <c r="AH7" s="76"/>
-      <c r="AI7" s="76"/>
-      <c r="AJ7" s="76"/>
-      <c r="AK7" s="76"/>
-      <c r="AL7" s="76"/>
-      <c r="AM7" s="76"/>
-      <c r="AN7" s="76"/>
-      <c r="AO7" s="76"/>
-      <c r="AP7" s="76"/>
-      <c r="AQ7" s="76"/>
-      <c r="AR7" s="76"/>
-      <c r="AS7" s="76"/>
-      <c r="AT7" s="76"/>
-      <c r="AU7" s="76"/>
-      <c r="AV7" s="77"/>
-      <c r="AW7" s="78"/>
-      <c r="AX7" s="79"/>
-      <c r="AY7" s="79"/>
-      <c r="AZ7" s="79"/>
-      <c r="BA7" s="79"/>
-      <c r="BB7" s="79"/>
-      <c r="BC7" s="79"/>
-      <c r="BD7" s="79"/>
-      <c r="BE7" s="79"/>
-      <c r="BF7" s="79"/>
-      <c r="BG7" s="79"/>
-      <c r="BH7" s="79"/>
-      <c r="BI7" s="79"/>
-      <c r="BJ7" s="79"/>
-      <c r="BK7" s="79"/>
-      <c r="BL7" s="79"/>
-      <c r="BM7" s="79"/>
-      <c r="BN7" s="79"/>
-      <c r="BO7" s="79"/>
-      <c r="BP7" s="80"/>
-      <c r="BQ7" s="81"/>
-      <c r="BR7" s="82"/>
-      <c r="BS7" s="82"/>
-      <c r="BT7" s="82"/>
-      <c r="BU7" s="82"/>
-      <c r="BV7" s="82"/>
-      <c r="BW7" s="82"/>
-      <c r="BX7" s="82"/>
-      <c r="BY7" s="82"/>
-      <c r="BZ7" s="82"/>
-      <c r="CA7" s="82"/>
-      <c r="CB7" s="82"/>
-      <c r="CC7" s="82"/>
-      <c r="CD7" s="82"/>
-      <c r="CE7" s="82"/>
-      <c r="CF7" s="82"/>
-      <c r="CG7" s="82"/>
-      <c r="CH7" s="82"/>
-      <c r="CI7" s="82"/>
-      <c r="CJ7" s="83"/>
-      <c r="CK7" s="84" t="s">
+      <c r="I7" s="84"/>
+      <c r="J7" s="85"/>
+      <c r="K7" s="85"/>
+      <c r="L7" s="85"/>
+      <c r="M7" s="85"/>
+      <c r="N7" s="85"/>
+      <c r="O7" s="85"/>
+      <c r="P7" s="85"/>
+      <c r="Q7" s="85"/>
+      <c r="R7" s="85"/>
+      <c r="S7" s="85"/>
+      <c r="T7" s="85"/>
+      <c r="U7" s="85"/>
+      <c r="V7" s="85"/>
+      <c r="W7" s="85"/>
+      <c r="X7" s="85"/>
+      <c r="Y7" s="85"/>
+      <c r="Z7" s="85"/>
+      <c r="AA7" s="85"/>
+      <c r="AB7" s="86"/>
+      <c r="AC7" s="89"/>
+      <c r="AD7" s="90"/>
+      <c r="AE7" s="90"/>
+      <c r="AF7" s="90"/>
+      <c r="AG7" s="90"/>
+      <c r="AH7" s="90"/>
+      <c r="AI7" s="90"/>
+      <c r="AJ7" s="90"/>
+      <c r="AK7" s="90"/>
+      <c r="AL7" s="90"/>
+      <c r="AM7" s="90"/>
+      <c r="AN7" s="90"/>
+      <c r="AO7" s="90"/>
+      <c r="AP7" s="90"/>
+      <c r="AQ7" s="90"/>
+      <c r="AR7" s="90"/>
+      <c r="AS7" s="90"/>
+      <c r="AT7" s="90"/>
+      <c r="AU7" s="90"/>
+      <c r="AV7" s="91"/>
+      <c r="AW7" s="94"/>
+      <c r="AX7" s="95"/>
+      <c r="AY7" s="95"/>
+      <c r="AZ7" s="95"/>
+      <c r="BA7" s="95"/>
+      <c r="BB7" s="95"/>
+      <c r="BC7" s="95"/>
+      <c r="BD7" s="95"/>
+      <c r="BE7" s="95"/>
+      <c r="BF7" s="95"/>
+      <c r="BG7" s="95"/>
+      <c r="BH7" s="95"/>
+      <c r="BI7" s="95"/>
+      <c r="BJ7" s="95"/>
+      <c r="BK7" s="95"/>
+      <c r="BL7" s="95"/>
+      <c r="BM7" s="95"/>
+      <c r="BN7" s="95"/>
+      <c r="BO7" s="95"/>
+      <c r="BP7" s="96"/>
+      <c r="BQ7" s="99"/>
+      <c r="BR7" s="100"/>
+      <c r="BS7" s="100"/>
+      <c r="BT7" s="100"/>
+      <c r="BU7" s="100"/>
+      <c r="BV7" s="100"/>
+      <c r="BW7" s="100"/>
+      <c r="BX7" s="100"/>
+      <c r="BY7" s="100"/>
+      <c r="BZ7" s="100"/>
+      <c r="CA7" s="100"/>
+      <c r="CB7" s="100"/>
+      <c r="CC7" s="100"/>
+      <c r="CD7" s="100"/>
+      <c r="CE7" s="100"/>
+      <c r="CF7" s="100"/>
+      <c r="CG7" s="100"/>
+      <c r="CH7" s="100"/>
+      <c r="CI7" s="100"/>
+      <c r="CJ7" s="101"/>
+      <c r="CK7" s="104" t="s">
         <v>52</v>
       </c>
-      <c r="CL7" s="85"/>
-      <c r="CM7" s="85"/>
-      <c r="CN7" s="85"/>
-      <c r="CO7" s="85"/>
+      <c r="CL7" s="105"/>
+      <c r="CM7" s="105"/>
+      <c r="CN7" s="105"/>
+      <c r="CO7" s="105"/>
       <c r="CP7" s="56"/>
     </row>
     <row r="8" spans="2:94" ht="27" x14ac:dyDescent="0.25">
@@ -2008,125 +2008,125 @@
       <c r="H8" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="63" t="s">
+      <c r="I8" s="87" t="s">
         <v>30</v>
       </c>
-      <c r="J8" s="64"/>
-      <c r="K8" s="64"/>
-      <c r="L8" s="64"/>
-      <c r="M8" s="64"/>
-      <c r="N8" s="63" t="s">
+      <c r="J8" s="88"/>
+      <c r="K8" s="88"/>
+      <c r="L8" s="88"/>
+      <c r="M8" s="88"/>
+      <c r="N8" s="87" t="s">
         <v>31</v>
       </c>
-      <c r="O8" s="64"/>
-      <c r="P8" s="64"/>
-      <c r="Q8" s="64"/>
-      <c r="R8" s="64"/>
-      <c r="S8" s="63" t="s">
+      <c r="O8" s="88"/>
+      <c r="P8" s="88"/>
+      <c r="Q8" s="88"/>
+      <c r="R8" s="88"/>
+      <c r="S8" s="87" t="s">
         <v>32</v>
       </c>
-      <c r="T8" s="64"/>
-      <c r="U8" s="64"/>
-      <c r="V8" s="64"/>
-      <c r="W8" s="64"/>
-      <c r="X8" s="63" t="s">
+      <c r="T8" s="88"/>
+      <c r="U8" s="88"/>
+      <c r="V8" s="88"/>
+      <c r="W8" s="88"/>
+      <c r="X8" s="87" t="s">
         <v>33</v>
       </c>
-      <c r="Y8" s="64"/>
-      <c r="Z8" s="64"/>
-      <c r="AA8" s="64"/>
-      <c r="AB8" s="64"/>
-      <c r="AC8" s="65" t="s">
+      <c r="Y8" s="88"/>
+      <c r="Z8" s="88"/>
+      <c r="AA8" s="88"/>
+      <c r="AB8" s="88"/>
+      <c r="AC8" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AD8" s="66"/>
-      <c r="AE8" s="66"/>
-      <c r="AF8" s="66"/>
-      <c r="AG8" s="66"/>
-      <c r="AH8" s="65" t="s">
+      <c r="AD8" s="93"/>
+      <c r="AE8" s="93"/>
+      <c r="AF8" s="93"/>
+      <c r="AG8" s="93"/>
+      <c r="AH8" s="92" t="s">
         <v>35</v>
       </c>
-      <c r="AI8" s="66"/>
-      <c r="AJ8" s="66"/>
-      <c r="AK8" s="66"/>
-      <c r="AL8" s="66"/>
-      <c r="AM8" s="65" t="s">
+      <c r="AI8" s="93"/>
+      <c r="AJ8" s="93"/>
+      <c r="AK8" s="93"/>
+      <c r="AL8" s="93"/>
+      <c r="AM8" s="92" t="s">
         <v>36</v>
       </c>
-      <c r="AN8" s="66"/>
-      <c r="AO8" s="66"/>
-      <c r="AP8" s="66"/>
-      <c r="AQ8" s="66"/>
-      <c r="AR8" s="65" t="s">
+      <c r="AN8" s="93"/>
+      <c r="AO8" s="93"/>
+      <c r="AP8" s="93"/>
+      <c r="AQ8" s="93"/>
+      <c r="AR8" s="92" t="s">
         <v>37</v>
       </c>
-      <c r="AS8" s="66"/>
-      <c r="AT8" s="66"/>
-      <c r="AU8" s="66"/>
-      <c r="AV8" s="66"/>
-      <c r="AW8" s="67" t="s">
+      <c r="AS8" s="93"/>
+      <c r="AT8" s="93"/>
+      <c r="AU8" s="93"/>
+      <c r="AV8" s="93"/>
+      <c r="AW8" s="97" t="s">
         <v>38</v>
       </c>
-      <c r="AX8" s="68"/>
-      <c r="AY8" s="68"/>
-      <c r="AZ8" s="68"/>
-      <c r="BA8" s="68"/>
-      <c r="BB8" s="67" t="s">
+      <c r="AX8" s="98"/>
+      <c r="AY8" s="98"/>
+      <c r="AZ8" s="98"/>
+      <c r="BA8" s="98"/>
+      <c r="BB8" s="97" t="s">
         <v>39</v>
       </c>
-      <c r="BC8" s="68"/>
-      <c r="BD8" s="68"/>
-      <c r="BE8" s="68"/>
-      <c r="BF8" s="68"/>
-      <c r="BG8" s="67" t="s">
+      <c r="BC8" s="98"/>
+      <c r="BD8" s="98"/>
+      <c r="BE8" s="98"/>
+      <c r="BF8" s="98"/>
+      <c r="BG8" s="97" t="s">
         <v>40</v>
       </c>
-      <c r="BH8" s="68"/>
-      <c r="BI8" s="68"/>
-      <c r="BJ8" s="68"/>
-      <c r="BK8" s="68"/>
-      <c r="BL8" s="67" t="s">
+      <c r="BH8" s="98"/>
+      <c r="BI8" s="98"/>
+      <c r="BJ8" s="98"/>
+      <c r="BK8" s="98"/>
+      <c r="BL8" s="97" t="s">
         <v>41</v>
       </c>
-      <c r="BM8" s="68"/>
-      <c r="BN8" s="68"/>
-      <c r="BO8" s="68"/>
-      <c r="BP8" s="68"/>
-      <c r="BQ8" s="61" t="s">
+      <c r="BM8" s="98"/>
+      <c r="BN8" s="98"/>
+      <c r="BO8" s="98"/>
+      <c r="BP8" s="98"/>
+      <c r="BQ8" s="102" t="s">
         <v>47</v>
       </c>
-      <c r="BR8" s="62"/>
-      <c r="BS8" s="62"/>
-      <c r="BT8" s="62"/>
-      <c r="BU8" s="62"/>
-      <c r="BV8" s="61" t="s">
+      <c r="BR8" s="103"/>
+      <c r="BS8" s="103"/>
+      <c r="BT8" s="103"/>
+      <c r="BU8" s="103"/>
+      <c r="BV8" s="102" t="s">
         <v>48</v>
       </c>
-      <c r="BW8" s="62"/>
-      <c r="BX8" s="62"/>
-      <c r="BY8" s="62"/>
-      <c r="BZ8" s="62"/>
-      <c r="CA8" s="61" t="s">
+      <c r="BW8" s="103"/>
+      <c r="BX8" s="103"/>
+      <c r="BY8" s="103"/>
+      <c r="BZ8" s="103"/>
+      <c r="CA8" s="102" t="s">
         <v>49</v>
       </c>
-      <c r="CB8" s="62"/>
-      <c r="CC8" s="62"/>
-      <c r="CD8" s="62"/>
-      <c r="CE8" s="62"/>
-      <c r="CF8" s="86" t="s">
+      <c r="CB8" s="103"/>
+      <c r="CC8" s="103"/>
+      <c r="CD8" s="103"/>
+      <c r="CE8" s="103"/>
+      <c r="CF8" s="106" t="s">
         <v>50</v>
       </c>
-      <c r="CG8" s="87"/>
-      <c r="CH8" s="87"/>
-      <c r="CI8" s="87"/>
-      <c r="CJ8" s="88"/>
-      <c r="CK8" s="69" t="s">
+      <c r="CG8" s="107"/>
+      <c r="CH8" s="107"/>
+      <c r="CI8" s="107"/>
+      <c r="CJ8" s="108"/>
+      <c r="CK8" s="81" t="s">
         <v>51</v>
       </c>
-      <c r="CL8" s="70"/>
-      <c r="CM8" s="70"/>
-      <c r="CN8" s="70"/>
-      <c r="CO8" s="71"/>
+      <c r="CL8" s="82"/>
+      <c r="CM8" s="82"/>
+      <c r="CN8" s="82"/>
+      <c r="CO8" s="83"/>
       <c r="CP8" s="57"/>
     </row>
     <row r="9" spans="2:94" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2409,72 +2409,72 @@
       <c r="CP9" s="54"/>
     </row>
     <row r="10" spans="2:94" s="60" customFormat="1" ht="20.100000000000001" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="89" t="s">
+      <c r="B10" s="61" t="s">
         <v>147</v>
       </c>
-      <c r="C10" s="91" t="s">
+      <c r="C10" s="63" t="s">
         <v>148</v>
       </c>
-      <c r="D10" s="92"/>
-      <c r="E10" s="93"/>
-      <c r="F10" s="94"/>
-      <c r="G10" s="95" t="str">
+      <c r="D10" s="64"/>
+      <c r="E10" s="65"/>
+      <c r="F10" s="66"/>
+      <c r="G10" s="67" t="str">
         <f>IF(F10-E10=0,"",F10-E10)</f>
         <v/>
       </c>
-      <c r="H10" s="96"/>
-      <c r="I10" s="104">
+      <c r="H10" s="68"/>
+      <c r="I10" s="76">
         <v>10</v>
       </c>
-      <c r="J10" s="105">
+      <c r="J10" s="77">
         <v>11</v>
       </c>
-      <c r="K10" s="105">
+      <c r="K10" s="77">
         <v>12</v>
       </c>
-      <c r="L10" s="105">
+      <c r="L10" s="77">
         <v>13</v>
       </c>
-      <c r="M10" s="105">
+      <c r="M10" s="77">
         <v>14</v>
       </c>
-      <c r="N10" s="105">
+      <c r="N10" s="77">
         <v>17</v>
       </c>
-      <c r="O10" s="105">
+      <c r="O10" s="77">
         <v>18</v>
       </c>
-      <c r="P10" s="105">
+      <c r="P10" s="77">
         <v>19</v>
       </c>
-      <c r="Q10" s="105">
+      <c r="Q10" s="77">
         <v>20</v>
       </c>
-      <c r="R10" s="105">
+      <c r="R10" s="77">
         <v>21</v>
       </c>
-      <c r="S10" s="104">
+      <c r="S10" s="76">
         <v>24</v>
       </c>
-      <c r="T10" s="105">
+      <c r="T10" s="77">
         <v>25</v>
       </c>
-      <c r="U10" s="105">
+      <c r="U10" s="77">
         <v>26</v>
       </c>
-      <c r="V10" s="105">
+      <c r="V10" s="77">
         <v>26.5757575757575</v>
       </c>
-      <c r="W10" s="105">
+      <c r="W10" s="77">
         <v>27.878787878787801</v>
       </c>
-      <c r="X10" s="105">
+      <c r="X10" s="77">
         <v>31</v>
       </c>
-      <c r="Y10" s="105"/>
-      <c r="Z10" s="105"/>
-      <c r="AA10" s="105"/>
-      <c r="AB10" s="105"/>
+      <c r="Y10" s="77"/>
+      <c r="Z10" s="77"/>
+      <c r="AA10" s="77"/>
+      <c r="AB10" s="77"/>
       <c r="AC10" s="59"/>
       <c r="AD10" s="58"/>
       <c r="AE10" s="58"/>
@@ -2543,34 +2543,34 @@
       <c r="CP10" s="59"/>
     </row>
     <row r="11" spans="2:94" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="90" t="s">
+      <c r="B11" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="99" t="s">
+      <c r="C11" s="71" t="s">
         <v>56</v>
       </c>
-      <c r="D11" s="99" t="s">
+      <c r="D11" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="E11" s="99" t="s">
+      <c r="E11" s="71" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="99" t="s">
+      <c r="F11" s="71" t="s">
         <v>58</v>
       </c>
-      <c r="G11" s="99" t="s">
+      <c r="G11" s="71" t="s">
         <v>59</v>
       </c>
-      <c r="H11" s="97">
+      <c r="H11" s="69">
         <v>1</v>
       </c>
-      <c r="I11" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="J11" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="K11" s="102" t="s">
+      <c r="I11" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="J11" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="K11" s="74" t="s">
         <v>149</v>
       </c>
       <c r="L11" s="21"/>
@@ -2658,40 +2658,40 @@
       <c r="CP11" s="20"/>
     </row>
     <row r="12" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="90" t="s">
+      <c r="B12" s="62" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="99" t="s">
+      <c r="C12" s="71" t="s">
         <v>60</v>
       </c>
-      <c r="D12" s="99" t="s">
+      <c r="D12" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="E12" s="99" t="s">
+      <c r="E12" s="71" t="s">
         <v>61</v>
       </c>
-      <c r="F12" s="99" t="s">
+      <c r="F12" s="71" t="s">
         <v>62</v>
       </c>
-      <c r="G12" s="99" t="s">
+      <c r="G12" s="71" t="s">
         <v>63</v>
       </c>
-      <c r="H12" s="97">
+      <c r="H12" s="69">
         <v>1</v>
       </c>
       <c r="I12" s="38"/>
       <c r="J12" s="21"/>
       <c r="K12" s="21"/>
-      <c r="L12" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="M12" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="N12" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="O12" s="106" t="s">
+      <c r="L12" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="M12" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="N12" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="O12" s="78" t="s">
         <v>149</v>
       </c>
       <c r="P12" s="22"/>
@@ -2775,26 +2775,26 @@
       <c r="CP12" s="20"/>
     </row>
     <row r="13" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="90" t="s">
+      <c r="B13" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="99" t="s">
+      <c r="C13" s="71" t="s">
         <v>64</v>
       </c>
-      <c r="D13" s="99" t="s">
+      <c r="D13" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="E13" s="99" t="s">
+      <c r="E13" s="71" t="s">
         <v>65</v>
       </c>
-      <c r="F13" s="99" t="s">
+      <c r="F13" s="71" t="s">
         <v>66</v>
       </c>
-      <c r="G13" s="99" t="s">
+      <c r="G13" s="71" t="s">
         <v>67</v>
       </c>
-      <c r="H13" s="97">
-        <v>0</v>
+      <c r="H13" s="69">
+        <v>1</v>
       </c>
       <c r="I13" s="38"/>
       <c r="J13" s="21"/>
@@ -2803,16 +2803,16 @@
       <c r="M13" s="21"/>
       <c r="N13" s="22"/>
       <c r="O13" s="22"/>
-      <c r="P13" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="Q13" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="R13" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="S13" s="102" t="s">
+      <c r="P13" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="Q13" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="R13" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="S13" s="74" t="s">
         <v>149</v>
       </c>
       <c r="T13" s="21"/>
@@ -2892,26 +2892,26 @@
       <c r="CP13" s="20"/>
     </row>
     <row r="14" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="90" t="s">
+      <c r="B14" s="62" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="99" t="s">
+      <c r="C14" s="71" t="s">
         <v>68</v>
       </c>
-      <c r="D14" s="99" t="s">
+      <c r="D14" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="E14" s="99" t="s">
+      <c r="E14" s="71" t="s">
         <v>65</v>
       </c>
-      <c r="F14" s="99" t="s">
+      <c r="F14" s="71" t="s">
         <v>69</v>
       </c>
-      <c r="G14" s="99" t="s">
+      <c r="G14" s="71" t="s">
         <v>63</v>
       </c>
-      <c r="H14" s="97">
-        <v>0</v>
+      <c r="H14" s="69">
+        <v>1</v>
       </c>
       <c r="I14" s="38"/>
       <c r="J14" s="21"/>
@@ -2920,19 +2920,19 @@
       <c r="M14" s="21"/>
       <c r="N14" s="22"/>
       <c r="O14" s="22"/>
-      <c r="P14" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="Q14" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="R14" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="S14" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="T14" s="102" t="s">
+      <c r="P14" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="Q14" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="R14" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="S14" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="T14" s="74" t="s">
         <v>149</v>
       </c>
       <c r="U14" s="21"/>
@@ -3011,26 +3011,26 @@
       <c r="CP14" s="20"/>
     </row>
     <row r="15" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="90" t="s">
+      <c r="B15" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="99" t="s">
+      <c r="C15" s="71" t="s">
         <v>70</v>
       </c>
-      <c r="D15" s="99" t="s">
+      <c r="D15" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="E15" s="99" t="s">
+      <c r="E15" s="71" t="s">
         <v>65</v>
       </c>
-      <c r="F15" s="99" t="s">
+      <c r="F15" s="71" t="s">
         <v>66</v>
       </c>
-      <c r="G15" s="99" t="s">
+      <c r="G15" s="71" t="s">
         <v>67</v>
       </c>
-      <c r="H15" s="97">
-        <v>0</v>
+      <c r="H15" s="69">
+        <v>1</v>
       </c>
       <c r="I15" s="38"/>
       <c r="J15" s="21"/>
@@ -3039,31 +3039,31 @@
       <c r="M15" s="21"/>
       <c r="N15" s="22"/>
       <c r="O15" s="22"/>
-      <c r="P15" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="Q15" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="R15" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="S15" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="T15" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="U15" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="V15" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="W15" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="X15" s="106" t="s">
+      <c r="P15" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="Q15" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="R15" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="S15" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="T15" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="U15" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="V15" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="W15" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="X15" s="78" t="s">
         <v>149</v>
       </c>
       <c r="Y15" s="22"/>
@@ -3138,26 +3138,26 @@
       <c r="CP15" s="20"/>
     </row>
     <row r="16" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="90" t="s">
+      <c r="B16" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="99" t="s">
+      <c r="C16" s="71" t="s">
         <v>71</v>
       </c>
-      <c r="D16" s="99" t="s">
+      <c r="D16" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="E16" s="99" t="s">
+      <c r="E16" s="71" t="s">
         <v>72</v>
       </c>
-      <c r="F16" s="99" t="s">
+      <c r="F16" s="71" t="s">
         <v>55</v>
       </c>
-      <c r="G16" s="99" t="s">
+      <c r="G16" s="71" t="s">
         <v>63</v>
       </c>
-      <c r="H16" s="97">
-        <v>0</v>
+      <c r="H16" s="69">
+        <v>0.5</v>
       </c>
       <c r="I16" s="38"/>
       <c r="J16" s="21"/>
@@ -3171,16 +3171,16 @@
       <c r="R16" s="22"/>
       <c r="S16" s="21"/>
       <c r="T16" s="21"/>
-      <c r="U16" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="V16" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="W16" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="X16" s="106" t="s">
+      <c r="U16" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="V16" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="W16" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="X16" s="78" t="s">
         <v>149</v>
       </c>
       <c r="Y16" s="22"/>
@@ -3255,25 +3255,25 @@
       <c r="CP16" s="20"/>
     </row>
     <row r="17" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="90" t="s">
+      <c r="B17" s="62" t="s">
         <v>73</v>
       </c>
-      <c r="C17" s="100" t="s">
+      <c r="C17" s="72" t="s">
         <v>74</v>
       </c>
-      <c r="D17" s="100" t="s">
+      <c r="D17" s="72" t="s">
         <v>57</v>
       </c>
-      <c r="E17" s="100" t="s">
+      <c r="E17" s="72" t="s">
         <v>55</v>
       </c>
-      <c r="F17" s="100" t="s">
+      <c r="F17" s="72" t="s">
         <v>55</v>
       </c>
-      <c r="G17" s="100" t="s">
+      <c r="G17" s="72" t="s">
         <v>150</v>
       </c>
-      <c r="H17" s="97">
+      <c r="H17" s="69">
         <v>0</v>
       </c>
       <c r="I17" s="38"/>
@@ -3291,13 +3291,13 @@
       <c r="U17" s="21"/>
       <c r="V17" s="21"/>
       <c r="W17" s="21"/>
-      <c r="X17" s="103" t="s">
+      <c r="X17" s="75" t="s">
         <v>149</v>
       </c>
       <c r="Y17" s="22"/>
       <c r="Z17" s="22"/>
       <c r="AA17" s="22"/>
-      <c r="AB17" s="103"/>
+      <c r="AB17" s="75"/>
       <c r="AC17" s="20"/>
       <c r="AD17" s="21"/>
       <c r="AE17" s="21"/>
@@ -3366,20 +3366,20 @@
       <c r="CP17" s="20"/>
     </row>
     <row r="18" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="90">
+      <c r="B18" s="62">
         <v>2</v>
       </c>
-      <c r="C18" s="101" t="s">
+      <c r="C18" s="73" t="s">
         <v>76</v>
       </c>
-      <c r="D18" s="92"/>
-      <c r="E18" s="93"/>
-      <c r="F18" s="94"/>
-      <c r="G18" s="95" t="str">
+      <c r="D18" s="64"/>
+      <c r="E18" s="65"/>
+      <c r="F18" s="66"/>
+      <c r="G18" s="67" t="str">
         <f>IF(F18-E18=0,"",F18-E18)</f>
         <v/>
       </c>
-      <c r="H18" s="96"/>
+      <c r="H18" s="68"/>
       <c r="I18" s="37"/>
       <c r="J18" s="19"/>
       <c r="K18" s="19"/>
@@ -3578,25 +3578,25 @@
       <c r="CP18" s="59"/>
     </row>
     <row r="19" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="90" t="s">
+      <c r="B19" s="62" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="99" t="s">
+      <c r="C19" s="71" t="s">
         <v>79</v>
       </c>
-      <c r="D19" s="99" t="s">
+      <c r="D19" s="71" t="s">
         <v>80</v>
       </c>
-      <c r="E19" s="99" t="s">
+      <c r="E19" s="71" t="s">
         <v>77</v>
       </c>
-      <c r="F19" s="99" t="s">
+      <c r="F19" s="71" t="s">
         <v>81</v>
       </c>
-      <c r="G19" s="99" t="s">
+      <c r="G19" s="71" t="s">
         <v>59</v>
       </c>
-      <c r="H19" s="97">
+      <c r="H19" s="69">
         <v>0</v>
       </c>
       <c r="I19" s="38"/>
@@ -3615,13 +3615,13 @@
       <c r="V19" s="21"/>
       <c r="W19" s="21"/>
       <c r="X19" s="22"/>
-      <c r="Y19" s="103" t="s">
-        <v>149</v>
-      </c>
-      <c r="Z19" s="103" t="s">
-        <v>149</v>
-      </c>
-      <c r="AA19" s="103" t="s">
+      <c r="Y19" s="75" t="s">
+        <v>149</v>
+      </c>
+      <c r="Z19" s="75" t="s">
+        <v>149</v>
+      </c>
+      <c r="AA19" s="75" t="s">
         <v>149</v>
       </c>
       <c r="AB19" s="22"/>
@@ -3693,25 +3693,25 @@
       <c r="CP19" s="20"/>
     </row>
     <row r="20" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="90" t="s">
+      <c r="B20" s="62" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="99" t="s">
+      <c r="C20" s="71" t="s">
         <v>82</v>
       </c>
-      <c r="D20" s="99" t="s">
+      <c r="D20" s="71" t="s">
         <v>80</v>
       </c>
-      <c r="E20" s="99" t="s">
+      <c r="E20" s="71" t="s">
         <v>83</v>
       </c>
-      <c r="F20" s="99" t="s">
+      <c r="F20" s="71" t="s">
         <v>84</v>
       </c>
-      <c r="G20" s="99" t="s">
+      <c r="G20" s="71" t="s">
         <v>63</v>
       </c>
-      <c r="H20" s="97">
+      <c r="H20" s="69">
         <v>0</v>
       </c>
       <c r="I20" s="38"/>
@@ -3732,17 +3732,17 @@
       <c r="X20" s="22"/>
       <c r="Y20" s="22"/>
       <c r="Z20" s="22"/>
-      <c r="AA20" s="103"/>
-      <c r="AB20" s="103" t="s">
-        <v>149</v>
-      </c>
-      <c r="AC20" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AD20" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AE20" s="102" t="s">
+      <c r="AA20" s="75"/>
+      <c r="AB20" s="75" t="s">
+        <v>149</v>
+      </c>
+      <c r="AC20" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AD20" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AE20" s="74" t="s">
         <v>149</v>
       </c>
       <c r="AF20" s="21"/>
@@ -3810,25 +3810,25 @@
       <c r="CP20" s="20"/>
     </row>
     <row r="21" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="90" t="s">
+      <c r="B21" s="62" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="99" t="s">
+      <c r="C21" s="71" t="s">
         <v>85</v>
       </c>
-      <c r="D21" s="99" t="s">
+      <c r="D21" s="71" t="s">
         <v>86</v>
       </c>
-      <c r="E21" s="99" t="s">
+      <c r="E21" s="71" t="s">
         <v>83</v>
       </c>
-      <c r="F21" s="99" t="s">
+      <c r="F21" s="71" t="s">
         <v>84</v>
       </c>
-      <c r="G21" s="99" t="s">
+      <c r="G21" s="71" t="s">
         <v>63</v>
       </c>
-      <c r="H21" s="97">
+      <c r="H21" s="69">
         <v>0</v>
       </c>
       <c r="I21" s="38"/>
@@ -3850,16 +3850,16 @@
       <c r="Y21" s="22"/>
       <c r="Z21" s="22"/>
       <c r="AA21" s="22"/>
-      <c r="AB21" s="103" t="s">
-        <v>149</v>
-      </c>
-      <c r="AC21" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AD21" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AE21" s="102" t="s">
+      <c r="AB21" s="75" t="s">
+        <v>149</v>
+      </c>
+      <c r="AC21" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AD21" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AE21" s="74" t="s">
         <v>149</v>
       </c>
       <c r="AF21" s="21"/>
@@ -3927,25 +3927,25 @@
       <c r="CP21" s="20"/>
     </row>
     <row r="22" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="90" t="s">
+      <c r="B22" s="62" t="s">
         <v>26</v>
       </c>
-      <c r="C22" s="99" t="s">
+      <c r="C22" s="71" t="s">
         <v>87</v>
       </c>
-      <c r="D22" s="99" t="s">
+      <c r="D22" s="71" t="s">
         <v>86</v>
       </c>
-      <c r="E22" s="99" t="s">
+      <c r="E22" s="71" t="s">
         <v>88</v>
       </c>
-      <c r="F22" s="99" t="s">
+      <c r="F22" s="71" t="s">
         <v>89</v>
       </c>
-      <c r="G22" s="99" t="s">
+      <c r="G22" s="71" t="s">
         <v>63</v>
       </c>
-      <c r="H22" s="97">
+      <c r="H22" s="69">
         <v>0</v>
       </c>
       <c r="I22" s="38"/>
@@ -3971,16 +3971,16 @@
       <c r="AC22" s="20"/>
       <c r="AD22" s="21"/>
       <c r="AE22" s="21"/>
-      <c r="AF22" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AG22" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AH22" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AI22" s="107" t="s">
+      <c r="AF22" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AG22" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AH22" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AI22" s="79" t="s">
         <v>149</v>
       </c>
       <c r="AJ22" s="23"/>
@@ -4044,25 +4044,25 @@
       <c r="CP22" s="20"/>
     </row>
     <row r="23" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="90" t="s">
+      <c r="B23" s="62" t="s">
         <v>90</v>
       </c>
-      <c r="C23" s="99" t="s">
+      <c r="C23" s="71" t="s">
         <v>91</v>
       </c>
-      <c r="D23" s="99" t="s">
+      <c r="D23" s="71" t="s">
         <v>80</v>
       </c>
-      <c r="E23" s="99" t="s">
+      <c r="E23" s="71" t="s">
         <v>88</v>
       </c>
-      <c r="F23" s="99" t="s">
+      <c r="F23" s="71" t="s">
         <v>92</v>
       </c>
-      <c r="G23" s="99" t="s">
+      <c r="G23" s="71" t="s">
         <v>93</v>
       </c>
-      <c r="H23" s="97">
+      <c r="H23" s="69">
         <v>0</v>
       </c>
       <c r="I23" s="38"/>
@@ -4088,49 +4088,49 @@
       <c r="AC23" s="20"/>
       <c r="AD23" s="21"/>
       <c r="AE23" s="21"/>
-      <c r="AF23" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AG23" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AH23" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AI23" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AJ23" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AK23" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AL23" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AM23" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AN23" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AO23" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AP23" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AQ23" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AR23" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AS23" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AT23" s="107" t="s">
+      <c r="AF23" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AG23" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AH23" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AI23" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AJ23" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AK23" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AL23" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AM23" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AN23" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AO23" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AP23" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AQ23" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AR23" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AS23" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AT23" s="79" t="s">
         <v>149</v>
       </c>
       <c r="AU23" s="23"/>
@@ -4183,25 +4183,25 @@
       <c r="CP23" s="20"/>
     </row>
     <row r="24" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="90" t="s">
+      <c r="B24" s="62" t="s">
         <v>94</v>
       </c>
-      <c r="C24" s="99" t="s">
+      <c r="C24" s="71" t="s">
         <v>95</v>
       </c>
-      <c r="D24" s="99" t="s">
+      <c r="D24" s="71" t="s">
         <v>80</v>
       </c>
-      <c r="E24" s="99" t="s">
+      <c r="E24" s="71" t="s">
         <v>96</v>
       </c>
-      <c r="F24" s="99" t="s">
+      <c r="F24" s="71" t="s">
         <v>97</v>
       </c>
-      <c r="G24" s="99" t="s">
+      <c r="G24" s="71" t="s">
         <v>98</v>
       </c>
-      <c r="H24" s="97">
+      <c r="H24" s="69">
         <v>0</v>
       </c>
       <c r="I24" s="38"/>
@@ -4242,34 +4242,34 @@
       <c r="AR24" s="23"/>
       <c r="AS24" s="23"/>
       <c r="AT24" s="23"/>
-      <c r="AU24" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AV24" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AW24" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AX24" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AY24" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AZ24" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BA24" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BB24" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BC24" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BD24" s="106" t="s">
+      <c r="AU24" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AV24" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AW24" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AX24" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AY24" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AZ24" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BA24" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BB24" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BC24" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BD24" s="78" t="s">
         <v>149</v>
       </c>
       <c r="BE24" s="22"/>
@@ -4312,25 +4312,25 @@
       <c r="CP24" s="20"/>
     </row>
     <row r="25" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="90" t="s">
+      <c r="B25" s="62" t="s">
         <v>99</v>
       </c>
-      <c r="C25" s="99" t="s">
+      <c r="C25" s="71" t="s">
         <v>100</v>
       </c>
-      <c r="D25" s="99" t="s">
+      <c r="D25" s="71" t="s">
         <v>80</v>
       </c>
-      <c r="E25" s="99" t="s">
+      <c r="E25" s="71" t="s">
         <v>96</v>
       </c>
-      <c r="F25" s="99" t="s">
+      <c r="F25" s="71" t="s">
         <v>97</v>
       </c>
-      <c r="G25" s="99" t="s">
+      <c r="G25" s="71" t="s">
         <v>98</v>
       </c>
-      <c r="H25" s="97">
+      <c r="H25" s="69">
         <v>0</v>
       </c>
       <c r="I25" s="38"/>
@@ -4371,34 +4371,34 @@
       <c r="AR25" s="23"/>
       <c r="AS25" s="23"/>
       <c r="AT25" s="23"/>
-      <c r="AU25" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AV25" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AW25" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AX25" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AY25" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AZ25" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BA25" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BB25" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BC25" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BD25" s="106" t="s">
+      <c r="AU25" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AV25" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AW25" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AX25" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AY25" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AZ25" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BA25" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BB25" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BC25" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BD25" s="78" t="s">
         <v>149</v>
       </c>
       <c r="BE25" s="22"/>
@@ -4441,25 +4441,25 @@
       <c r="CP25" s="20"/>
     </row>
     <row r="26" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="90" t="s">
+      <c r="B26" s="62" t="s">
         <v>101</v>
       </c>
-      <c r="C26" s="99" t="s">
+      <c r="C26" s="71" t="s">
         <v>102</v>
       </c>
-      <c r="D26" s="99" t="s">
+      <c r="D26" s="71" t="s">
         <v>86</v>
       </c>
-      <c r="E26" s="99" t="s">
+      <c r="E26" s="71" t="s">
         <v>96</v>
       </c>
-      <c r="F26" s="99" t="s">
+      <c r="F26" s="71" t="s">
         <v>97</v>
       </c>
-      <c r="G26" s="99" t="s">
+      <c r="G26" s="71" t="s">
         <v>98</v>
       </c>
-      <c r="H26" s="97">
+      <c r="H26" s="69">
         <v>0</v>
       </c>
       <c r="I26" s="38"/>
@@ -4500,34 +4500,34 @@
       <c r="AR26" s="23"/>
       <c r="AS26" s="23"/>
       <c r="AT26" s="23"/>
-      <c r="AU26" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AV26" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AW26" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AX26" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AY26" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AZ26" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BA26" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BB26" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BC26" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BD26" s="106" t="s">
+      <c r="AU26" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AV26" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AW26" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AX26" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AY26" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AZ26" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BA26" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BB26" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BC26" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BD26" s="78" t="s">
         <v>149</v>
       </c>
       <c r="BE26" s="22"/>
@@ -4570,25 +4570,25 @@
       <c r="CP26" s="20"/>
     </row>
     <row r="27" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="90" t="s">
+      <c r="B27" s="62" t="s">
         <v>103</v>
       </c>
-      <c r="C27" s="99" t="s">
+      <c r="C27" s="71" t="s">
         <v>104</v>
       </c>
-      <c r="D27" s="99" t="s">
+      <c r="D27" s="71" t="s">
         <v>86</v>
       </c>
-      <c r="E27" s="99" t="s">
+      <c r="E27" s="71" t="s">
         <v>96</v>
       </c>
-      <c r="F27" s="99" t="s">
+      <c r="F27" s="71" t="s">
         <v>97</v>
       </c>
-      <c r="G27" s="99" t="s">
+      <c r="G27" s="71" t="s">
         <v>98</v>
       </c>
-      <c r="H27" s="97">
+      <c r="H27" s="69">
         <v>0</v>
       </c>
       <c r="I27" s="38"/>
@@ -4629,34 +4629,34 @@
       <c r="AR27" s="23"/>
       <c r="AS27" s="23"/>
       <c r="AT27" s="23"/>
-      <c r="AU27" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AV27" s="107" t="s">
-        <v>149</v>
-      </c>
-      <c r="AW27" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AX27" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AY27" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="AZ27" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BA27" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BB27" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BC27" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BD27" s="106" t="s">
+      <c r="AU27" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AV27" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="AW27" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AX27" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AY27" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="AZ27" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BA27" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BB27" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BC27" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BD27" s="78" t="s">
         <v>149</v>
       </c>
       <c r="BE27" s="22"/>
@@ -4699,25 +4699,25 @@
       <c r="CP27" s="20"/>
     </row>
     <row r="28" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="90" t="s">
+      <c r="B28" s="62" t="s">
         <v>105</v>
       </c>
-      <c r="C28" s="99" t="s">
+      <c r="C28" s="71" t="s">
         <v>106</v>
       </c>
-      <c r="D28" s="99" t="s">
+      <c r="D28" s="71" t="s">
         <v>86</v>
       </c>
-      <c r="E28" s="99" t="s">
+      <c r="E28" s="71" t="s">
         <v>107</v>
       </c>
-      <c r="F28" s="99" t="s">
+      <c r="F28" s="71" t="s">
         <v>108</v>
       </c>
-      <c r="G28" s="99" t="s">
+      <c r="G28" s="71" t="s">
         <v>67</v>
       </c>
-      <c r="H28" s="97">
+      <c r="H28" s="69">
         <v>0</v>
       </c>
       <c r="I28" s="38"/>
@@ -4768,19 +4768,19 @@
       <c r="BB28" s="22"/>
       <c r="BC28" s="22"/>
       <c r="BD28" s="22"/>
-      <c r="BE28" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BF28" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BG28" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BH28" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BI28" s="102" t="s">
+      <c r="BE28" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BF28" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BG28" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BH28" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BI28" s="74" t="s">
         <v>149</v>
       </c>
       <c r="BJ28" s="21"/>
@@ -4818,25 +4818,25 @@
       <c r="CP28" s="20"/>
     </row>
     <row r="29" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="90" t="s">
+      <c r="B29" s="62" t="s">
         <v>109</v>
       </c>
-      <c r="C29" s="99" t="s">
+      <c r="C29" s="71" t="s">
         <v>110</v>
       </c>
-      <c r="D29" s="99" t="s">
+      <c r="D29" s="71" t="s">
         <v>80</v>
       </c>
-      <c r="E29" s="99" t="s">
+      <c r="E29" s="71" t="s">
         <v>107</v>
       </c>
-      <c r="F29" s="99" t="s">
+      <c r="F29" s="71" t="s">
         <v>111</v>
       </c>
-      <c r="G29" s="99" t="s">
+      <c r="G29" s="71" t="s">
         <v>63</v>
       </c>
-      <c r="H29" s="97">
+      <c r="H29" s="69">
         <v>0</v>
       </c>
       <c r="I29" s="38"/>
@@ -4887,19 +4887,19 @@
       <c r="BB29" s="22"/>
       <c r="BC29" s="22"/>
       <c r="BD29" s="22"/>
-      <c r="BE29" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BF29" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BG29" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BH29" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BI29" s="102"/>
+      <c r="BE29" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BF29" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BG29" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BH29" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BI29" s="74"/>
       <c r="BJ29" s="21"/>
       <c r="BK29" s="21"/>
       <c r="BL29" s="22"/>
@@ -4935,25 +4935,25 @@
       <c r="CP29" s="20"/>
     </row>
     <row r="30" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="90" t="s">
+      <c r="B30" s="62" t="s">
         <v>112</v>
       </c>
-      <c r="C30" s="99" t="s">
+      <c r="C30" s="71" t="s">
         <v>113</v>
       </c>
-      <c r="D30" s="99" t="s">
+      <c r="D30" s="71" t="s">
         <v>80</v>
       </c>
-      <c r="E30" s="99" t="s">
+      <c r="E30" s="71" t="s">
         <v>107</v>
       </c>
-      <c r="F30" s="99" t="s">
+      <c r="F30" s="71" t="s">
         <v>111</v>
       </c>
-      <c r="G30" s="99" t="s">
+      <c r="G30" s="71" t="s">
         <v>63</v>
       </c>
-      <c r="H30" s="97">
+      <c r="H30" s="69">
         <v>0</v>
       </c>
       <c r="I30" s="38"/>
@@ -5004,16 +5004,16 @@
       <c r="BB30" s="22"/>
       <c r="BC30" s="22"/>
       <c r="BD30" s="22"/>
-      <c r="BE30" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BF30" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BG30" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BH30" s="102" t="s">
+      <c r="BE30" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BF30" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BG30" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BH30" s="74" t="s">
         <v>149</v>
       </c>
       <c r="BI30" s="21"/>
@@ -5052,25 +5052,25 @@
       <c r="CP30" s="20"/>
     </row>
     <row r="31" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="90" t="s">
+      <c r="B31" s="62" t="s">
         <v>114</v>
       </c>
-      <c r="C31" s="99" t="s">
+      <c r="C31" s="71" t="s">
         <v>115</v>
       </c>
-      <c r="D31" s="99" t="s">
+      <c r="D31" s="71" t="s">
         <v>80</v>
       </c>
-      <c r="E31" s="99" t="s">
+      <c r="E31" s="71" t="s">
         <v>116</v>
       </c>
-      <c r="F31" s="99" t="s">
+      <c r="F31" s="71" t="s">
         <v>117</v>
       </c>
-      <c r="G31" s="99" t="s">
+      <c r="G31" s="71" t="s">
         <v>118</v>
       </c>
-      <c r="H31" s="97">
+      <c r="H31" s="69">
         <v>0</v>
       </c>
       <c r="I31" s="38"/>
@@ -5124,32 +5124,32 @@
       <c r="BE31" s="22"/>
       <c r="BF31" s="22"/>
       <c r="BG31" s="21"/>
-      <c r="BI31" s="102"/>
-      <c r="BJ31" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BK31" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BL31" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BM31" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BN31" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BO31" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BP31" s="106" t="s">
-        <v>149</v>
-      </c>
-      <c r="BQ31" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BR31" s="102" t="s">
+      <c r="BI31" s="74"/>
+      <c r="BJ31" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BK31" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BL31" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BM31" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BN31" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BO31" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BP31" s="78" t="s">
+        <v>149</v>
+      </c>
+      <c r="BQ31" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BR31" s="74" t="s">
         <v>149</v>
       </c>
       <c r="BS31" s="21"/>
@@ -5178,25 +5178,25 @@
       <c r="CP31" s="20"/>
     </row>
     <row r="32" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="90" t="s">
+      <c r="B32" s="62" t="s">
         <v>119</v>
       </c>
-      <c r="C32" s="99" t="s">
+      <c r="C32" s="71" t="s">
         <v>120</v>
       </c>
-      <c r="D32" s="99" t="s">
+      <c r="D32" s="71" t="s">
         <v>86</v>
       </c>
-      <c r="E32" s="99" t="s">
+      <c r="E32" s="71" t="s">
         <v>121</v>
       </c>
-      <c r="F32" s="99" t="s">
+      <c r="F32" s="71" t="s">
         <v>122</v>
       </c>
-      <c r="G32" s="99" t="s">
+      <c r="G32" s="71" t="s">
         <v>123</v>
       </c>
-      <c r="H32" s="97">
+      <c r="H32" s="69">
         <v>0</v>
       </c>
       <c r="I32" s="38"/>
@@ -5261,25 +5261,25 @@
       <c r="BP32" s="22"/>
       <c r="BQ32" s="20"/>
       <c r="BR32" s="21"/>
-      <c r="BS32" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BT32" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BU32" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BV32" s="108" t="s">
-        <v>149</v>
-      </c>
-      <c r="BW32" s="108" t="s">
-        <v>149</v>
-      </c>
-      <c r="BX32" s="108" t="s">
-        <v>149</v>
-      </c>
-      <c r="BY32" s="108" t="s">
+      <c r="BS32" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BT32" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BU32" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BV32" s="80" t="s">
+        <v>149</v>
+      </c>
+      <c r="BW32" s="80" t="s">
+        <v>149</v>
+      </c>
+      <c r="BX32" s="80" t="s">
+        <v>149</v>
+      </c>
+      <c r="BY32" s="80" t="s">
         <v>149</v>
       </c>
       <c r="BZ32" s="24"/>
@@ -5301,25 +5301,25 @@
       <c r="CP32" s="20"/>
     </row>
     <row r="33" spans="2:94" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="90" t="s">
+      <c r="B33" s="62" t="s">
         <v>124</v>
       </c>
-      <c r="C33" s="99" t="s">
+      <c r="C33" s="71" t="s">
         <v>125</v>
       </c>
-      <c r="D33" s="99" t="s">
+      <c r="D33" s="71" t="s">
         <v>86</v>
       </c>
-      <c r="E33" s="99" t="s">
+      <c r="E33" s="71" t="s">
         <v>126</v>
       </c>
-      <c r="F33" s="99" t="s">
+      <c r="F33" s="71" t="s">
         <v>127</v>
       </c>
-      <c r="G33" s="99" t="s">
+      <c r="G33" s="71" t="s">
         <v>59</v>
       </c>
-      <c r="H33" s="98">
+      <c r="H33" s="70">
         <v>0</v>
       </c>
       <c r="I33" s="38"/>
@@ -5365,13 +5365,13 @@
       <c r="AW33" s="20"/>
       <c r="AX33" s="21"/>
       <c r="AY33" s="21"/>
-      <c r="AZ33" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BA33" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="BB33" s="106" t="s">
+      <c r="AZ33" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BA33" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="BB33" s="78" t="s">
         <v>149</v>
       </c>
       <c r="BC33" s="22"/>
@@ -5416,25 +5416,25 @@
       <c r="CP33" s="20"/>
     </row>
     <row r="34" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="90" t="s">
+      <c r="B34" s="62" t="s">
         <v>128</v>
       </c>
-      <c r="C34" s="100" t="s">
+      <c r="C34" s="72" t="s">
         <v>129</v>
       </c>
-      <c r="D34" s="100" t="s">
+      <c r="D34" s="72" t="s">
         <v>57</v>
       </c>
-      <c r="E34" s="100" t="s">
+      <c r="E34" s="72" t="s">
         <v>127</v>
       </c>
-      <c r="F34" s="100" t="s">
+      <c r="F34" s="72" t="s">
         <v>127</v>
       </c>
-      <c r="G34" s="100" t="s">
+      <c r="G34" s="72" t="s">
         <v>75</v>
       </c>
-      <c r="H34" s="97">
+      <c r="H34" s="69">
         <v>0</v>
       </c>
       <c r="I34" s="38"/>
@@ -5482,7 +5482,7 @@
       <c r="AY34" s="21"/>
       <c r="AZ34" s="21"/>
       <c r="BA34" s="21"/>
-      <c r="BB34" s="106" t="s">
+      <c r="BB34" s="78" t="s">
         <v>149</v>
       </c>
       <c r="BC34" s="22"/>
@@ -5527,25 +5527,25 @@
       <c r="CP34" s="20"/>
     </row>
     <row r="35" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="90" t="s">
+      <c r="B35" s="62" t="s">
         <v>130</v>
       </c>
-      <c r="C35" s="99" t="s">
+      <c r="C35" s="71" t="s">
         <v>131</v>
       </c>
-      <c r="D35" s="99" t="s">
+      <c r="D35" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="E35" s="99" t="s">
+      <c r="E35" s="71" t="s">
         <v>132</v>
       </c>
-      <c r="F35" s="99" t="s">
+      <c r="F35" s="71" t="s">
         <v>78</v>
       </c>
-      <c r="G35" s="99" t="s">
+      <c r="G35" s="71" t="s">
         <v>133</v>
       </c>
-      <c r="H35" s="97">
+      <c r="H35" s="69">
         <v>0</v>
       </c>
       <c r="I35" s="38"/>
@@ -5617,10 +5617,10 @@
       <c r="BW35" s="24"/>
       <c r="BX35" s="24"/>
       <c r="BY35" s="24"/>
-      <c r="BZ35" s="108" t="s">
-        <v>149</v>
-      </c>
-      <c r="CA35" s="102" t="s">
+      <c r="BZ35" s="80" t="s">
+        <v>149</v>
+      </c>
+      <c r="CA35" s="74" t="s">
         <v>149</v>
       </c>
       <c r="CB35" s="21"/>
@@ -5640,25 +5640,25 @@
       <c r="CP35" s="20"/>
     </row>
     <row r="36" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="90" t="s">
+      <c r="B36" s="62" t="s">
         <v>134</v>
       </c>
-      <c r="C36" s="100" t="s">
+      <c r="C36" s="72" t="s">
         <v>135</v>
       </c>
-      <c r="D36" s="100" t="s">
+      <c r="D36" s="72" t="s">
         <v>57</v>
       </c>
-      <c r="E36" s="100" t="s">
+      <c r="E36" s="72" t="s">
         <v>78</v>
       </c>
-      <c r="F36" s="100" t="s">
+      <c r="F36" s="72" t="s">
         <v>78</v>
       </c>
-      <c r="G36" s="100" t="s">
+      <c r="G36" s="72" t="s">
         <v>75</v>
       </c>
-      <c r="H36" s="97">
+      <c r="H36" s="69">
         <v>0</v>
       </c>
       <c r="I36" s="38"/>
@@ -5731,7 +5731,7 @@
       <c r="BX36" s="24"/>
       <c r="BY36" s="24"/>
       <c r="BZ36" s="24"/>
-      <c r="CA36" s="102" t="s">
+      <c r="CA36" s="74" t="s">
         <v>149</v>
       </c>
       <c r="CB36" s="21"/>
@@ -5751,17 +5751,17 @@
       <c r="CP36" s="20"/>
     </row>
     <row r="37" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="90">
+      <c r="B37" s="62">
         <v>3</v>
       </c>
-      <c r="C37" s="101" t="s">
+      <c r="C37" s="73" t="s">
         <v>136</v>
       </c>
-      <c r="D37" s="96"/>
-      <c r="E37" s="96"/>
-      <c r="F37" s="96"/>
-      <c r="G37" s="96"/>
-      <c r="H37" s="96"/>
+      <c r="D37" s="68"/>
+      <c r="E37" s="68"/>
+      <c r="F37" s="68"/>
+      <c r="G37" s="68"/>
+      <c r="H37" s="68"/>
       <c r="I37" s="37"/>
       <c r="J37" s="19"/>
       <c r="K37" s="19"/>
@@ -5880,25 +5880,25 @@
       </c>
     </row>
     <row r="38" spans="2:94" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="90" t="s">
+      <c r="B38" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="C38" s="99" t="s">
+      <c r="C38" s="71" t="s">
         <v>139</v>
       </c>
-      <c r="D38" s="99" t="s">
+      <c r="D38" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="E38" s="99" t="s">
+      <c r="E38" s="71" t="s">
         <v>137</v>
       </c>
-      <c r="F38" s="99" t="s">
+      <c r="F38" s="71" t="s">
         <v>140</v>
       </c>
-      <c r="G38" s="99" t="s">
+      <c r="G38" s="71" t="s">
         <v>67</v>
       </c>
-      <c r="H38" s="98">
+      <c r="H38" s="70">
         <v>0</v>
       </c>
       <c r="I38" s="39"/>
@@ -5972,19 +5972,19 @@
       <c r="BY38" s="29"/>
       <c r="BZ38" s="29"/>
       <c r="CA38" s="26"/>
-      <c r="CB38" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="CC38" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="CD38" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="CE38" s="102" t="s">
-        <v>149</v>
-      </c>
-      <c r="CF38" s="108" t="s">
+      <c r="CB38" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="CC38" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="CD38" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="CE38" s="74" t="s">
+        <v>149</v>
+      </c>
+      <c r="CF38" s="80" t="s">
         <v>149</v>
       </c>
       <c r="CG38" s="29"/>
@@ -5999,25 +5999,25 @@
       <c r="CP38" s="25"/>
     </row>
     <row r="39" spans="2:94" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B39" s="90" t="s">
+      <c r="B39" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="C39" s="99" t="s">
+      <c r="C39" s="71" t="s">
         <v>141</v>
       </c>
-      <c r="D39" s="99" t="s">
+      <c r="D39" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="E39" s="99" t="s">
+      <c r="E39" s="71" t="s">
         <v>140</v>
       </c>
-      <c r="F39" s="99" t="s">
+      <c r="F39" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="G39" s="99" t="s">
+      <c r="G39" s="71" t="s">
         <v>67</v>
       </c>
-      <c r="H39" s="97">
+      <c r="H39" s="69">
         <v>0</v>
       </c>
       <c r="I39" s="38"/>
@@ -6095,19 +6095,19 @@
       <c r="CC39" s="21"/>
       <c r="CD39" s="21"/>
       <c r="CE39" s="21"/>
-      <c r="CF39" s="108" t="s">
-        <v>149</v>
-      </c>
-      <c r="CG39" s="108" t="s">
-        <v>149</v>
-      </c>
-      <c r="CH39" s="108" t="s">
-        <v>149</v>
-      </c>
-      <c r="CI39" s="108" t="s">
-        <v>149</v>
-      </c>
-      <c r="CJ39" s="108" t="s">
+      <c r="CF39" s="80" t="s">
+        <v>149</v>
+      </c>
+      <c r="CG39" s="80" t="s">
+        <v>149</v>
+      </c>
+      <c r="CH39" s="80" t="s">
+        <v>149</v>
+      </c>
+      <c r="CI39" s="80" t="s">
+        <v>149</v>
+      </c>
+      <c r="CJ39" s="80" t="s">
         <v>149</v>
       </c>
       <c r="CK39" s="20"/>
@@ -6118,25 +6118,25 @@
       <c r="CP39" s="20"/>
     </row>
     <row r="40" spans="2:94" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B40" s="90" t="s">
+      <c r="B40" s="62" t="s">
         <v>29</v>
       </c>
-      <c r="C40" s="99" t="s">
+      <c r="C40" s="71" t="s">
         <v>143</v>
       </c>
-      <c r="D40" s="99" t="s">
+      <c r="D40" s="71" t="s">
         <v>57</v>
       </c>
-      <c r="E40" s="99" t="s">
+      <c r="E40" s="71" t="s">
         <v>144</v>
       </c>
-      <c r="F40" s="99" t="s">
+      <c r="F40" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="G40" s="99" t="s">
+      <c r="G40" s="71" t="s">
         <v>63</v>
       </c>
-      <c r="H40" s="97">
+      <c r="H40" s="69">
         <v>0</v>
       </c>
       <c r="I40" s="38"/>
@@ -6215,45 +6215,45 @@
       <c r="CD40" s="21"/>
       <c r="CE40" s="21"/>
       <c r="CF40" s="24"/>
-      <c r="CG40" s="108" t="s">
-        <v>149</v>
-      </c>
-      <c r="CH40" s="108" t="s">
-        <v>149</v>
-      </c>
-      <c r="CI40" s="108" t="s">
-        <v>149</v>
-      </c>
-      <c r="CJ40" s="108" t="s">
-        <v>149</v>
-      </c>
-      <c r="CK40" s="102"/>
+      <c r="CG40" s="80" t="s">
+        <v>149</v>
+      </c>
+      <c r="CH40" s="80" t="s">
+        <v>149</v>
+      </c>
+      <c r="CI40" s="80" t="s">
+        <v>149</v>
+      </c>
+      <c r="CJ40" s="80" t="s">
+        <v>149</v>
+      </c>
+      <c r="CK40" s="74"/>
       <c r="CL40" s="21"/>
       <c r="CM40" s="21"/>
       <c r="CN40" s="21"/>
       <c r="CO40" s="21"/>
       <c r="CP40" s="20"/>
     </row>
-    <row r="41" spans="2:94" ht="27" x14ac:dyDescent="0.25">
-      <c r="B41" s="90" t="s">
+    <row r="41" spans="2:94" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="B41" s="62" t="s">
         <v>145</v>
       </c>
-      <c r="C41" s="100" t="s">
+      <c r="C41" s="72" t="s">
         <v>146</v>
       </c>
-      <c r="D41" s="100" t="s">
+      <c r="D41" s="72" t="s">
         <v>57</v>
       </c>
-      <c r="E41" s="100" t="s">
+      <c r="E41" s="72" t="s">
         <v>138</v>
       </c>
-      <c r="F41" s="100" t="s">
+      <c r="F41" s="72" t="s">
         <v>138</v>
       </c>
-      <c r="G41" s="100" t="s">
+      <c r="G41" s="72" t="s">
         <v>75</v>
       </c>
-      <c r="H41" s="97">
+      <c r="H41" s="69">
         <v>0</v>
       </c>
       <c r="I41" s="38"/>
@@ -6341,7 +6341,7 @@
       <c r="CM41" s="21"/>
       <c r="CN41" s="21"/>
       <c r="CO41" s="21"/>
-      <c r="CP41" s="102" t="s">
+      <c r="CP41" s="74" t="s">
         <v>149</v>
       </c>
     </row>
@@ -6350,6 +6350,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="BV8:BZ8"/>
+    <mergeCell ref="S8:W8"/>
+    <mergeCell ref="AC8:AG8"/>
+    <mergeCell ref="AH8:AL8"/>
+    <mergeCell ref="AR8:AV8"/>
+    <mergeCell ref="AW8:BA8"/>
     <mergeCell ref="CK8:CO8"/>
     <mergeCell ref="I7:AB7"/>
     <mergeCell ref="X8:AB8"/>
@@ -6366,14 +6372,22 @@
     <mergeCell ref="BB8:BF8"/>
     <mergeCell ref="BL8:BP8"/>
     <mergeCell ref="BQ8:BU8"/>
-    <mergeCell ref="BV8:BZ8"/>
-    <mergeCell ref="S8:W8"/>
-    <mergeCell ref="AC8:AG8"/>
-    <mergeCell ref="AH8:AL8"/>
-    <mergeCell ref="AR8:AV8"/>
-    <mergeCell ref="AW8:BA8"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
+  <conditionalFormatting sqref="D37:G37">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="percent" val="0"/>
+        <cfvo type="percent" val="100"/>
+        <color theme="3" tint="0.59999389629810485"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{92566078-8F6F-41ED-8B2D-AE8E56452D11}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H10:H41">
     <cfRule type="dataBar" priority="3">
       <dataBar>
@@ -6388,25 +6402,26 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D37:G37">
-    <cfRule type="dataBar" priority="1">
-      <dataBar>
-        <cfvo type="percent" val="0"/>
-        <cfvo type="percent" val="100"/>
-        <color theme="3" tint="0.59999389629810485"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{92566078-8F6F-41ED-8B2D-AE8E56452D11}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{92566078-8F6F-41ED-8B2D-AE8E56452D11}">
+            <x14:dataBar minLength="0" maxLength="100">
+              <x14:cfvo type="percent">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="percent">
+                <xm:f>100</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor theme="0"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D37:G37</xm:sqref>
+        </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{FE5B685F-D93A-1B44-AB73-D05D527007CF}">
             <x14:dataBar minLength="0" maxLength="100">
@@ -6422,21 +6437,6 @@
           </x14:cfRule>
           <xm:sqref>H10:H41</xm:sqref>
         </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{92566078-8F6F-41ED-8B2D-AE8E56452D11}">
-            <x14:dataBar minLength="0" maxLength="100">
-              <x14:cfvo type="percent">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="percent">
-                <xm:f>100</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor theme="0"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D37:G37</xm:sqref>
-        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
   </extLst>

</xml_diff>

<commit_message>
Mejorar visualización del dashboard operacional
- Incorporación de anillos de progreso para cumplimiento de servicios y pasajeros.
- Implementación de gráfico doughnut para distribución de estados de servicios.
- Implementación de gráfico doughnut para composición de personas transportadas.
- Reorganización de desviaciones operacionales en una card compacta.
- Incorporación de leyendas y valores visibles en los gráficos circulares.
- Definición de paleta semántica reutilizable para estados operacionales.
- Uso consistente de colores para planificados, en curso, realizados, cancelados y no planificados.
- Manejo visual de períodos sin servicios o personas transportadas.
- Ajustes de componentes compartidos para mantener alturas y composición uniforme.
- Integración de los nuevos gráficos con los filtros existentes del dashboard.
- Sin nuevos endpoints ni modificaciones al backend.
- Build de Angular verificado correctamente.
</commit_message>
<xml_diff>
--- a/FASE 1/Evidencias Grupales/Gantt CAPSTONE - SISTEMA DE GESTION PARA TRANSPORTE DE PASAJEROS.xlsx
+++ b/FASE 1/Evidencias Grupales/Gantt CAPSTONE - SISTEMA DE GESTION PARA TRANSPORTE DE PASAJEROS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\capstone-2026\FASE 1\Evidencias Grupales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A15E728A-1C2A-447F-A5BD-C1AED8BD3F5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32D5B373-F735-4516-A216-8CD2DEB8FD36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gestión Proyecto Carta Gantt" sheetId="3" r:id="rId1"/>
@@ -498,7 +498,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1512,73 +1512,73 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="22" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1822,7 +1822,7 @@
     <tabColor theme="3" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="B1:CP45"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.875" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.5" customWidth="1"/>
     <col min="2" max="2" width="14.625" customWidth="1"/>
@@ -1836,7 +1836,7 @@
     <col min="94" max="94" width="2.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:94" s="34" customFormat="1" ht="50.1" customHeight="1">
+    <row r="1" spans="2:94" s="34" customFormat="1" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="35" t="s">
         <v>0</v>
       </c>
@@ -1858,7 +1858,7 @@
       <c r="R1" s="36"/>
       <c r="S1" s="36"/>
     </row>
-    <row r="2" spans="2:94" s="1" customFormat="1" ht="35.1" customHeight="1">
+    <row r="2" spans="2:94" s="1" customFormat="1" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="44" t="s">
         <v>1</v>
       </c>
@@ -1866,19 +1866,19 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="2:94" s="1" customFormat="1" ht="27.75" thickBot="1">
+    <row r="3" spans="2:94" s="1" customFormat="1" ht="27.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="47" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="48"/>
     </row>
-    <row r="4" spans="2:94" s="1" customFormat="1" ht="27.75" thickTop="1">
+    <row r="4" spans="2:94" s="1" customFormat="1" ht="27.75" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B4" s="46" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="43"/>
     </row>
-    <row r="5" spans="2:94" s="1" customFormat="1" ht="17.25">
+    <row r="5" spans="2:94" s="1" customFormat="1" ht="17.25" x14ac:dyDescent="0.3">
       <c r="B5" s="45" t="s">
         <v>4</v>
       </c>
@@ -1886,10 +1886,10 @@
         <v>46255</v>
       </c>
     </row>
-    <row r="6" spans="2:94" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1">
+    <row r="6" spans="2:94" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="2"/>
     </row>
-    <row r="7" spans="2:94" ht="20.100000000000001" customHeight="1" thickBot="1">
+    <row r="7" spans="2:94" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="4"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
@@ -1897,86 +1897,86 @@
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
-      <c r="I7" s="92"/>
-      <c r="J7" s="93"/>
-      <c r="K7" s="93"/>
-      <c r="L7" s="93"/>
-      <c r="M7" s="93"/>
-      <c r="N7" s="93"/>
-      <c r="O7" s="93"/>
-      <c r="P7" s="93"/>
-      <c r="Q7" s="93"/>
-      <c r="R7" s="93"/>
-      <c r="S7" s="93"/>
-      <c r="T7" s="93"/>
-      <c r="U7" s="93"/>
-      <c r="V7" s="93"/>
-      <c r="W7" s="93"/>
-      <c r="X7" s="93"/>
-      <c r="Y7" s="93"/>
-      <c r="Z7" s="93"/>
-      <c r="AA7" s="93"/>
-      <c r="AB7" s="94"/>
-      <c r="AC7" s="95"/>
-      <c r="AD7" s="96"/>
-      <c r="AE7" s="96"/>
-      <c r="AF7" s="96"/>
-      <c r="AG7" s="96"/>
-      <c r="AH7" s="96"/>
-      <c r="AI7" s="96"/>
-      <c r="AJ7" s="96"/>
-      <c r="AK7" s="96"/>
-      <c r="AL7" s="96"/>
-      <c r="AM7" s="96"/>
-      <c r="AN7" s="96"/>
-      <c r="AO7" s="96"/>
-      <c r="AP7" s="96"/>
-      <c r="AQ7" s="96"/>
-      <c r="AR7" s="96"/>
-      <c r="AS7" s="96"/>
-      <c r="AT7" s="96"/>
-      <c r="AU7" s="96"/>
-      <c r="AV7" s="97"/>
-      <c r="AW7" s="98"/>
-      <c r="AX7" s="99"/>
-      <c r="AY7" s="99"/>
-      <c r="AZ7" s="99"/>
-      <c r="BA7" s="99"/>
-      <c r="BB7" s="99"/>
-      <c r="BC7" s="99"/>
-      <c r="BD7" s="99"/>
-      <c r="BE7" s="99"/>
-      <c r="BF7" s="99"/>
-      <c r="BG7" s="99"/>
-      <c r="BH7" s="99"/>
-      <c r="BI7" s="99"/>
-      <c r="BJ7" s="99"/>
-      <c r="BK7" s="99"/>
-      <c r="BL7" s="99"/>
-      <c r="BM7" s="99"/>
-      <c r="BN7" s="99"/>
-      <c r="BO7" s="99"/>
-      <c r="BP7" s="100"/>
-      <c r="BQ7" s="101"/>
-      <c r="BR7" s="102"/>
-      <c r="BS7" s="102"/>
-      <c r="BT7" s="102"/>
-      <c r="BU7" s="102"/>
-      <c r="BV7" s="102"/>
-      <c r="BW7" s="102"/>
-      <c r="BX7" s="102"/>
-      <c r="BY7" s="102"/>
-      <c r="BZ7" s="102"/>
-      <c r="CA7" s="102"/>
-      <c r="CB7" s="102"/>
-      <c r="CC7" s="102"/>
-      <c r="CD7" s="102"/>
-      <c r="CE7" s="102"/>
-      <c r="CF7" s="102"/>
-      <c r="CG7" s="102"/>
-      <c r="CH7" s="102"/>
-      <c r="CI7" s="102"/>
-      <c r="CJ7" s="103"/>
+      <c r="I7" s="84"/>
+      <c r="J7" s="85"/>
+      <c r="K7" s="85"/>
+      <c r="L7" s="85"/>
+      <c r="M7" s="85"/>
+      <c r="N7" s="85"/>
+      <c r="O7" s="85"/>
+      <c r="P7" s="85"/>
+      <c r="Q7" s="85"/>
+      <c r="R7" s="85"/>
+      <c r="S7" s="85"/>
+      <c r="T7" s="85"/>
+      <c r="U7" s="85"/>
+      <c r="V7" s="85"/>
+      <c r="W7" s="85"/>
+      <c r="X7" s="85"/>
+      <c r="Y7" s="85"/>
+      <c r="Z7" s="85"/>
+      <c r="AA7" s="85"/>
+      <c r="AB7" s="86"/>
+      <c r="AC7" s="89"/>
+      <c r="AD7" s="90"/>
+      <c r="AE7" s="90"/>
+      <c r="AF7" s="90"/>
+      <c r="AG7" s="90"/>
+      <c r="AH7" s="90"/>
+      <c r="AI7" s="90"/>
+      <c r="AJ7" s="90"/>
+      <c r="AK7" s="90"/>
+      <c r="AL7" s="90"/>
+      <c r="AM7" s="90"/>
+      <c r="AN7" s="90"/>
+      <c r="AO7" s="90"/>
+      <c r="AP7" s="90"/>
+      <c r="AQ7" s="90"/>
+      <c r="AR7" s="90"/>
+      <c r="AS7" s="90"/>
+      <c r="AT7" s="90"/>
+      <c r="AU7" s="90"/>
+      <c r="AV7" s="91"/>
+      <c r="AW7" s="94"/>
+      <c r="AX7" s="95"/>
+      <c r="AY7" s="95"/>
+      <c r="AZ7" s="95"/>
+      <c r="BA7" s="95"/>
+      <c r="BB7" s="95"/>
+      <c r="BC7" s="95"/>
+      <c r="BD7" s="95"/>
+      <c r="BE7" s="95"/>
+      <c r="BF7" s="95"/>
+      <c r="BG7" s="95"/>
+      <c r="BH7" s="95"/>
+      <c r="BI7" s="95"/>
+      <c r="BJ7" s="95"/>
+      <c r="BK7" s="95"/>
+      <c r="BL7" s="95"/>
+      <c r="BM7" s="95"/>
+      <c r="BN7" s="95"/>
+      <c r="BO7" s="95"/>
+      <c r="BP7" s="96"/>
+      <c r="BQ7" s="99"/>
+      <c r="BR7" s="100"/>
+      <c r="BS7" s="100"/>
+      <c r="BT7" s="100"/>
+      <c r="BU7" s="100"/>
+      <c r="BV7" s="100"/>
+      <c r="BW7" s="100"/>
+      <c r="BX7" s="100"/>
+      <c r="BY7" s="100"/>
+      <c r="BZ7" s="100"/>
+      <c r="CA7" s="100"/>
+      <c r="CB7" s="100"/>
+      <c r="CC7" s="100"/>
+      <c r="CD7" s="100"/>
+      <c r="CE7" s="100"/>
+      <c r="CF7" s="100"/>
+      <c r="CG7" s="100"/>
+      <c r="CH7" s="100"/>
+      <c r="CI7" s="100"/>
+      <c r="CJ7" s="101"/>
       <c r="CK7" s="104" t="s">
         <v>52</v>
       </c>
@@ -1986,7 +1986,7 @@
       <c r="CO7" s="105"/>
       <c r="CP7" s="56"/>
     </row>
-    <row r="8" spans="2:94" ht="27">
+    <row r="8" spans="2:94" ht="27" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
         <v>5</v>
       </c>
@@ -2008,111 +2008,111 @@
       <c r="H8" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="83" t="s">
+      <c r="I8" s="87" t="s">
         <v>30</v>
       </c>
-      <c r="J8" s="84"/>
-      <c r="K8" s="84"/>
-      <c r="L8" s="84"/>
-      <c r="M8" s="84"/>
-      <c r="N8" s="83" t="s">
+      <c r="J8" s="88"/>
+      <c r="K8" s="88"/>
+      <c r="L8" s="88"/>
+      <c r="M8" s="88"/>
+      <c r="N8" s="87" t="s">
         <v>31</v>
       </c>
-      <c r="O8" s="84"/>
-      <c r="P8" s="84"/>
-      <c r="Q8" s="84"/>
-      <c r="R8" s="84"/>
-      <c r="S8" s="83" t="s">
+      <c r="O8" s="88"/>
+      <c r="P8" s="88"/>
+      <c r="Q8" s="88"/>
+      <c r="R8" s="88"/>
+      <c r="S8" s="87" t="s">
         <v>32</v>
       </c>
-      <c r="T8" s="84"/>
-      <c r="U8" s="84"/>
-      <c r="V8" s="84"/>
-      <c r="W8" s="84"/>
-      <c r="X8" s="83" t="s">
+      <c r="T8" s="88"/>
+      <c r="U8" s="88"/>
+      <c r="V8" s="88"/>
+      <c r="W8" s="88"/>
+      <c r="X8" s="87" t="s">
         <v>33</v>
       </c>
-      <c r="Y8" s="84"/>
-      <c r="Z8" s="84"/>
-      <c r="AA8" s="84"/>
-      <c r="AB8" s="84"/>
-      <c r="AC8" s="85" t="s">
+      <c r="Y8" s="88"/>
+      <c r="Z8" s="88"/>
+      <c r="AA8" s="88"/>
+      <c r="AB8" s="88"/>
+      <c r="AC8" s="92" t="s">
         <v>34</v>
       </c>
-      <c r="AD8" s="86"/>
-      <c r="AE8" s="86"/>
-      <c r="AF8" s="86"/>
-      <c r="AG8" s="86"/>
-      <c r="AH8" s="85" t="s">
+      <c r="AD8" s="93"/>
+      <c r="AE8" s="93"/>
+      <c r="AF8" s="93"/>
+      <c r="AG8" s="93"/>
+      <c r="AH8" s="92" t="s">
         <v>35</v>
       </c>
-      <c r="AI8" s="86"/>
-      <c r="AJ8" s="86"/>
-      <c r="AK8" s="86"/>
-      <c r="AL8" s="86"/>
-      <c r="AM8" s="85" t="s">
+      <c r="AI8" s="93"/>
+      <c r="AJ8" s="93"/>
+      <c r="AK8" s="93"/>
+      <c r="AL8" s="93"/>
+      <c r="AM8" s="92" t="s">
         <v>36</v>
       </c>
-      <c r="AN8" s="86"/>
-      <c r="AO8" s="86"/>
-      <c r="AP8" s="86"/>
-      <c r="AQ8" s="86"/>
-      <c r="AR8" s="85" t="s">
+      <c r="AN8" s="93"/>
+      <c r="AO8" s="93"/>
+      <c r="AP8" s="93"/>
+      <c r="AQ8" s="93"/>
+      <c r="AR8" s="92" t="s">
         <v>37</v>
       </c>
-      <c r="AS8" s="86"/>
-      <c r="AT8" s="86"/>
-      <c r="AU8" s="86"/>
-      <c r="AV8" s="86"/>
-      <c r="AW8" s="87" t="s">
+      <c r="AS8" s="93"/>
+      <c r="AT8" s="93"/>
+      <c r="AU8" s="93"/>
+      <c r="AV8" s="93"/>
+      <c r="AW8" s="97" t="s">
         <v>38</v>
       </c>
-      <c r="AX8" s="88"/>
-      <c r="AY8" s="88"/>
-      <c r="AZ8" s="88"/>
-      <c r="BA8" s="88"/>
-      <c r="BB8" s="87" t="s">
+      <c r="AX8" s="98"/>
+      <c r="AY8" s="98"/>
+      <c r="AZ8" s="98"/>
+      <c r="BA8" s="98"/>
+      <c r="BB8" s="97" t="s">
         <v>39</v>
       </c>
-      <c r="BC8" s="88"/>
-      <c r="BD8" s="88"/>
-      <c r="BE8" s="88"/>
-      <c r="BF8" s="88"/>
-      <c r="BG8" s="87" t="s">
+      <c r="BC8" s="98"/>
+      <c r="BD8" s="98"/>
+      <c r="BE8" s="98"/>
+      <c r="BF8" s="98"/>
+      <c r="BG8" s="97" t="s">
         <v>40</v>
       </c>
-      <c r="BH8" s="88"/>
-      <c r="BI8" s="88"/>
-      <c r="BJ8" s="88"/>
-      <c r="BK8" s="88"/>
-      <c r="BL8" s="87" t="s">
+      <c r="BH8" s="98"/>
+      <c r="BI8" s="98"/>
+      <c r="BJ8" s="98"/>
+      <c r="BK8" s="98"/>
+      <c r="BL8" s="97" t="s">
         <v>41</v>
       </c>
-      <c r="BM8" s="88"/>
-      <c r="BN8" s="88"/>
-      <c r="BO8" s="88"/>
-      <c r="BP8" s="88"/>
-      <c r="BQ8" s="81" t="s">
+      <c r="BM8" s="98"/>
+      <c r="BN8" s="98"/>
+      <c r="BO8" s="98"/>
+      <c r="BP8" s="98"/>
+      <c r="BQ8" s="102" t="s">
         <v>47</v>
       </c>
-      <c r="BR8" s="82"/>
-      <c r="BS8" s="82"/>
-      <c r="BT8" s="82"/>
-      <c r="BU8" s="82"/>
-      <c r="BV8" s="81" t="s">
+      <c r="BR8" s="103"/>
+      <c r="BS8" s="103"/>
+      <c r="BT8" s="103"/>
+      <c r="BU8" s="103"/>
+      <c r="BV8" s="102" t="s">
         <v>48</v>
       </c>
-      <c r="BW8" s="82"/>
-      <c r="BX8" s="82"/>
-      <c r="BY8" s="82"/>
-      <c r="BZ8" s="82"/>
-      <c r="CA8" s="81" t="s">
+      <c r="BW8" s="103"/>
+      <c r="BX8" s="103"/>
+      <c r="BY8" s="103"/>
+      <c r="BZ8" s="103"/>
+      <c r="CA8" s="102" t="s">
         <v>49</v>
       </c>
-      <c r="CB8" s="82"/>
-      <c r="CC8" s="82"/>
-      <c r="CD8" s="82"/>
-      <c r="CE8" s="82"/>
+      <c r="CB8" s="103"/>
+      <c r="CC8" s="103"/>
+      <c r="CD8" s="103"/>
+      <c r="CE8" s="103"/>
       <c r="CF8" s="106" t="s">
         <v>50</v>
       </c>
@@ -2120,16 +2120,16 @@
       <c r="CH8" s="107"/>
       <c r="CI8" s="107"/>
       <c r="CJ8" s="108"/>
-      <c r="CK8" s="89" t="s">
+      <c r="CK8" s="81" t="s">
         <v>51</v>
       </c>
-      <c r="CL8" s="90"/>
-      <c r="CM8" s="90"/>
-      <c r="CN8" s="90"/>
-      <c r="CO8" s="91"/>
+      <c r="CL8" s="82"/>
+      <c r="CM8" s="82"/>
+      <c r="CN8" s="82"/>
+      <c r="CO8" s="83"/>
       <c r="CP8" s="57"/>
     </row>
-    <row r="9" spans="2:94" ht="20.100000000000001" customHeight="1" thickBot="1">
+    <row r="9" spans="2:94" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="9" t="s">
         <v>6</v>
       </c>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="CP9" s="54"/>
     </row>
-    <row r="10" spans="2:94" s="60" customFormat="1" ht="20.100000000000001" customHeight="1" thickTop="1">
+    <row r="10" spans="2:94" s="60" customFormat="1" ht="20.100000000000001" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B10" s="61" t="s">
         <v>147</v>
       </c>
@@ -2542,7 +2542,7 @@
       <c r="CO10" s="58"/>
       <c r="CP10" s="59"/>
     </row>
-    <row r="11" spans="2:94" ht="19.5" customHeight="1">
+    <row r="11" spans="2:94" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="62" t="s">
         <v>17</v>
       </c>
@@ -2657,7 +2657,7 @@
       <c r="CO11" s="21"/>
       <c r="CP11" s="20"/>
     </row>
-    <row r="12" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="12" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="62" t="s">
         <v>18</v>
       </c>
@@ -2774,7 +2774,7 @@
       <c r="CO12" s="21"/>
       <c r="CP12" s="20"/>
     </row>
-    <row r="13" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="13" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="62" t="s">
         <v>19</v>
       </c>
@@ -2891,7 +2891,7 @@
       <c r="CO13" s="21"/>
       <c r="CP13" s="20"/>
     </row>
-    <row r="14" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="14" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="62" t="s">
         <v>20</v>
       </c>
@@ -3010,7 +3010,7 @@
       <c r="CO14" s="21"/>
       <c r="CP14" s="20"/>
     </row>
-    <row r="15" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="15" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="62" t="s">
         <v>21</v>
       </c>
@@ -3137,7 +3137,7 @@
       <c r="CO15" s="21"/>
       <c r="CP15" s="20"/>
     </row>
-    <row r="16" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="16" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="62" t="s">
         <v>22</v>
       </c>
@@ -3157,7 +3157,7 @@
         <v>63</v>
       </c>
       <c r="H16" s="69">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="I16" s="38"/>
       <c r="J16" s="21"/>
@@ -3254,7 +3254,7 @@
       <c r="CO16" s="21"/>
       <c r="CP16" s="20"/>
     </row>
-    <row r="17" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="17" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="62" t="s">
         <v>73</v>
       </c>
@@ -3274,7 +3274,7 @@
         <v>150</v>
       </c>
       <c r="H17" s="69">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I17" s="38"/>
       <c r="J17" s="21"/>
@@ -3365,7 +3365,7 @@
       <c r="CO17" s="21"/>
       <c r="CP17" s="20"/>
     </row>
-    <row r="18" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="18" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="62">
         <v>2</v>
       </c>
@@ -3577,7 +3577,7 @@
       <c r="CO18" s="19"/>
       <c r="CP18" s="59"/>
     </row>
-    <row r="19" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="19" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="62" t="s">
         <v>23</v>
       </c>
@@ -3597,7 +3597,7 @@
         <v>59</v>
       </c>
       <c r="H19" s="69">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" s="38"/>
       <c r="J19" s="21"/>
@@ -3692,7 +3692,7 @@
       <c r="CO19" s="21"/>
       <c r="CP19" s="20"/>
     </row>
-    <row r="20" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="20" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="62" t="s">
         <v>24</v>
       </c>
@@ -3712,7 +3712,7 @@
         <v>63</v>
       </c>
       <c r="H20" s="69">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I20" s="38"/>
       <c r="J20" s="21"/>
@@ -3809,7 +3809,7 @@
       <c r="CO20" s="21"/>
       <c r="CP20" s="20"/>
     </row>
-    <row r="21" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="21" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="62" t="s">
         <v>25</v>
       </c>
@@ -3829,7 +3829,7 @@
         <v>63</v>
       </c>
       <c r="H21" s="69">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21" s="38"/>
       <c r="J21" s="21"/>
@@ -3926,7 +3926,7 @@
       <c r="CO21" s="21"/>
       <c r="CP21" s="20"/>
     </row>
-    <row r="22" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="22" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="62" t="s">
         <v>26</v>
       </c>
@@ -3946,7 +3946,7 @@
         <v>63</v>
       </c>
       <c r="H22" s="69">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I22" s="38"/>
       <c r="J22" s="21"/>
@@ -4043,7 +4043,7 @@
       <c r="CO22" s="21"/>
       <c r="CP22" s="20"/>
     </row>
-    <row r="23" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="23" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="62" t="s">
         <v>90</v>
       </c>
@@ -4063,7 +4063,7 @@
         <v>93</v>
       </c>
       <c r="H23" s="69">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="I23" s="38"/>
       <c r="J23" s="21"/>
@@ -4182,7 +4182,7 @@
       <c r="CO23" s="21"/>
       <c r="CP23" s="20"/>
     </row>
-    <row r="24" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="24" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="62" t="s">
         <v>94</v>
       </c>
@@ -4311,7 +4311,7 @@
       <c r="CO24" s="21"/>
       <c r="CP24" s="20"/>
     </row>
-    <row r="25" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="25" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="62" t="s">
         <v>99</v>
       </c>
@@ -4440,7 +4440,7 @@
       <c r="CO25" s="21"/>
       <c r="CP25" s="20"/>
     </row>
-    <row r="26" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="26" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="62" t="s">
         <v>101</v>
       </c>
@@ -4569,7 +4569,7 @@
       <c r="CO26" s="21"/>
       <c r="CP26" s="20"/>
     </row>
-    <row r="27" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="27" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="62" t="s">
         <v>103</v>
       </c>
@@ -4698,7 +4698,7 @@
       <c r="CO27" s="21"/>
       <c r="CP27" s="20"/>
     </row>
-    <row r="28" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="28" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="62" t="s">
         <v>105</v>
       </c>
@@ -4817,7 +4817,7 @@
       <c r="CO28" s="21"/>
       <c r="CP28" s="20"/>
     </row>
-    <row r="29" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="29" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="62" t="s">
         <v>109</v>
       </c>
@@ -4934,7 +4934,7 @@
       <c r="CO29" s="21"/>
       <c r="CP29" s="20"/>
     </row>
-    <row r="30" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="30" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="62" t="s">
         <v>112</v>
       </c>
@@ -5051,7 +5051,7 @@
       <c r="CO30" s="21"/>
       <c r="CP30" s="20"/>
     </row>
-    <row r="31" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="31" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="62" t="s">
         <v>114</v>
       </c>
@@ -5177,7 +5177,7 @@
       <c r="CO31" s="21"/>
       <c r="CP31" s="20"/>
     </row>
-    <row r="32" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="32" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="62" t="s">
         <v>119</v>
       </c>
@@ -5300,7 +5300,7 @@
       <c r="CO32" s="21"/>
       <c r="CP32" s="20"/>
     </row>
-    <row r="33" spans="2:94" ht="20.100000000000001" customHeight="1" thickBot="1">
+    <row r="33" spans="2:94" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="62" t="s">
         <v>124</v>
       </c>
@@ -5415,7 +5415,7 @@
       <c r="CO33" s="21"/>
       <c r="CP33" s="20"/>
     </row>
-    <row r="34" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="34" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="62" t="s">
         <v>128</v>
       </c>
@@ -5526,7 +5526,7 @@
       <c r="CO34" s="21"/>
       <c r="CP34" s="20"/>
     </row>
-    <row r="35" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="35" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="62" t="s">
         <v>130</v>
       </c>
@@ -5639,7 +5639,7 @@
       <c r="CO35" s="21"/>
       <c r="CP35" s="20"/>
     </row>
-    <row r="36" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="36" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="62" t="s">
         <v>134</v>
       </c>
@@ -5750,7 +5750,7 @@
       <c r="CO36" s="21"/>
       <c r="CP36" s="20"/>
     </row>
-    <row r="37" spans="2:94" ht="20.100000000000001" customHeight="1">
+    <row r="37" spans="2:94" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="62">
         <v>3</v>
       </c>
@@ -5879,7 +5879,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="2:94" ht="20.100000000000001" customHeight="1" thickBot="1">
+    <row r="38" spans="2:94" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B38" s="62" t="s">
         <v>27</v>
       </c>
@@ -5998,7 +5998,7 @@
       <c r="CO38" s="26"/>
       <c r="CP38" s="25"/>
     </row>
-    <row r="39" spans="2:94" ht="16.5">
+    <row r="39" spans="2:94" ht="16.5" x14ac:dyDescent="0.25">
       <c r="B39" s="62" t="s">
         <v>28</v>
       </c>
@@ -6117,7 +6117,7 @@
       <c r="CO39" s="21"/>
       <c r="CP39" s="20"/>
     </row>
-    <row r="40" spans="2:94" ht="16.5">
+    <row r="40" spans="2:94" ht="16.5" x14ac:dyDescent="0.25">
       <c r="B40" s="62" t="s">
         <v>29</v>
       </c>
@@ -6234,7 +6234,7 @@
       <c r="CO40" s="21"/>
       <c r="CP40" s="20"/>
     </row>
-    <row r="41" spans="2:94" ht="16.5">
+    <row r="41" spans="2:94" ht="16.5" x14ac:dyDescent="0.25">
       <c r="B41" s="62" t="s">
         <v>145</v>
       </c>
@@ -6345,11 +6345,17 @@
         <v>149</v>
       </c>
     </row>
-    <row r="45" spans="2:94" ht="19.5">
+    <row r="45" spans="2:94" ht="19.5" x14ac:dyDescent="0.3">
       <c r="C45" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="BV8:BZ8"/>
+    <mergeCell ref="S8:W8"/>
+    <mergeCell ref="AC8:AG8"/>
+    <mergeCell ref="AH8:AL8"/>
+    <mergeCell ref="AR8:AV8"/>
+    <mergeCell ref="AW8:BA8"/>
     <mergeCell ref="CK8:CO8"/>
     <mergeCell ref="I7:AB7"/>
     <mergeCell ref="X8:AB8"/>
@@ -6366,12 +6372,6 @@
     <mergeCell ref="BB8:BF8"/>
     <mergeCell ref="BL8:BP8"/>
     <mergeCell ref="BQ8:BU8"/>
-    <mergeCell ref="BV8:BZ8"/>
-    <mergeCell ref="S8:W8"/>
-    <mergeCell ref="AC8:AG8"/>
-    <mergeCell ref="AH8:AL8"/>
-    <mergeCell ref="AR8:AV8"/>
-    <mergeCell ref="AW8:BA8"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <conditionalFormatting sqref="D37:G37">

</xml_diff>